<commit_message>
Hogar de Refugio: análisis de ubicación rehecho para el hogar (condiciones propias del servicio)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/MATRIZ_INCOMPATIBILIDADES_UBICACION_HOGAR_REFUGIO.xlsx
+++ b/entregables/MATRIZ_INCOMPATIBILIDADES_UBICACION_HOGAR_REFUGIO.xlsx
@@ -10,7 +10,8 @@
   <sheets>
     <sheet name="MATRIZ" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="AREA DE INFLUENCIA" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="RESUMEN" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="CONDICIONES HOGAR" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="RESUMEN" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="121">
   <si>
     <t xml:space="preserve">MATRIZ DE INCOMPATIBILIDADES DE UBICACIÓN (CUADRO DE LA R.V.M. N.° 010-2022-MINEDU)</t>
   </si>
@@ -72,7 +73,7 @@
     <t xml:space="preserve">R.M. N.° 045-2015/MINSA, NTS N.° 113-MINSA/DGIEM-V.01 "Infraestructura y equipamiento de los establecimientos de salud del Primer Nivel de Atención", y R.M. N.° 862-2015/MINSA, NTS N.° 119-MINSA/DGIEM-V.01 "Infraestructura y equipamiento de los establecimientos de salud del Tercer Nivel de Atención"</t>
   </si>
   <si>
-    <t xml:space="preserve">El establecimiento de salud de la localidad se encuentra a más de 100 m del predio.</t>
+    <t xml:space="preserve">El establecimiento de salud de la localidad se encuentra a más de 100 m del predio y forma parte de los servicios de apoyo cercanos que requiere el hogar.</t>
   </si>
   <si>
     <t xml:space="preserve">Plantas envasadoras de gas licuado de petróleo (GLP)</t>
@@ -99,7 +100,7 @@
     <t xml:space="preserve">Ley N.° 28681, Ley que regula la comercialización, consumo y publicidad de bebidas alcohólicas, y su Reglamento (D.S. N.° 012-2009-SA)</t>
   </si>
   <si>
-    <t xml:space="preserve">No existen locales de venta y consumo de bebidas alcohólicas a menos de 100 m del predio.</t>
+    <t xml:space="preserve">No existen locales de venta y consumo de bebidas alcohólicas a menos de 100 m del predio, lo que favorece la tranquilidad y la seguridad de las residentes.</t>
   </si>
   <si>
     <t xml:space="preserve">Plantas de abastecimiento de combustibles líquidos y otros productos derivados de los hidrocarburos</t>
@@ -249,7 +250,7 @@
     <t xml:space="preserve">Zonificación y licencias municipales</t>
   </si>
   <si>
-    <t xml:space="preserve">No existen hostales, peñas, discotecas, video-pubs, bingos ni salas de billar en el entorno del predio.</t>
+    <t xml:space="preserve">No existen hostales, peñas, discotecas, video-pubs, bingos ni salas de billar en el entorno del predio; el entorno es tranquilo, como lo requiere un hogar de refugio.</t>
   </si>
   <si>
     <t xml:space="preserve">ÁREA DE INFLUENCIA MEDIDA DESDE EL LINDERO</t>
@@ -273,22 +274,115 @@
     <t xml:space="preserve">Fajas marginales de las fuentes de agua, naturales o artificiales; Pozos para la exploración y explotación de hidrocarburos; Aeródromos; Servidumbre de líneas aéreas de instalaciones eléctricas; Servidumbre de electroductos; Restricciones radioeléctricas en áreas de uso público próximas a una estación radioeléctrica; Plantas de tratamiento de aguas residuales; Faja de terreno lateral y colindante al derecho de vía; Zonas restringidas colindantes a las vías ferroviarias; Casinos y máquinas tragamonedas; Hostales, peñas, discotecas, video-pubs, bingos y salas de billar</t>
   </si>
   <si>
-    <t xml:space="preserve">RESUMEN DEL ANÁLISIS DE INCOMPATIBILIDADES</t>
+    <t xml:space="preserve">CONDICIONES DE UBICACIÓN PROPIAS DEL HOGAR DE REFUGIO TEMPORAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONDICIÓN DE UBICACIÓN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FUENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿EL PREDIO O EL PROYECTO LA SATISFACE?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CÓMO LA CUMPLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ubicación en zona compatible con la zonificación vigente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNE A.090, art. 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SÍ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predio rural Los Mangos, de propiedad del Gobierno Regional, destinado a servicios de protección social del Estado junto con el CAR Varones y el CAR Mujeres.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zona tranquila y no aislada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lineamientos ONU-Habitat / CONAVIM, num. 2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entorno urbano de Morales y Tarapoto, con frente a la carretera Oasis y colindante con otros servicios de protección; sin bares, discotecas ni casinos en el entorno (Cuadro N.° 1, filas 5, 17 y 18).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servicios e instituciones de apoyo cercanos (salud, seguridad y justicia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lineamientos, num. 2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servicios de salud, seguridad y justicia del distrito de Morales y de la ciudad de Tarapoto en el entorno urbano; el establecimiento de salud de la localidad está a más de 100 m (Cuadro N.° 1, fila 2).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accesos vehicular y peatonal, sin estudio de impacto vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lineamientos, num. 2.1 y 2.6; RNE A.090, art. 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acceso por la carretera Oasis, con ingreso principal y de servicio controlados. La población del hogar es menor de 500 personas, por lo que la A.090 (art. 4) no exige estudio de impacto vial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguridad frente a agresiones externas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lineamientos, num. 2.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recinto con cerco perimétrico, caseta de control en los accesos y cuarto de cámaras del circuito cerrado de vigilancia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserva del uso y privacidad de las residentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lineamientos, num. 2.2 y 2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conjunto de edificaciones dentro de un recinto cercado, sin anuncios que revelen el uso; los predios colindantes son servicios del Estado de acceso restringido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servicios básicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lineamientos, num. 2.8; RNE A.040, art. 7 d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El proyecto contempla cisterna y tanque elevado, tratamiento de aguas residuales, subestación eléctrica, grupo electrógeno y drenaje pluvial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protección frente a lluvias intensas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNE OS.060 (drenaje pluvial urbano)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drenaje pluvial del predio con colector frontal y cunetas, dimensionado con la hidrología del expediente; las obras quedan dentro del lindero.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESUMEN DEL ANÁLISIS DE UBICACIÓN</t>
   </si>
   <si>
     <t xml:space="preserve">CONCEPTO</t>
   </si>
   <si>
-    <t xml:space="preserve">CANTIDAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incompatibilidades evaluadas</t>
+    <t xml:space="preserve">EVALUADOS</t>
   </si>
   <si>
     <t xml:space="preserve">CUMPLE</t>
   </si>
   <si>
     <t xml:space="preserve">NO CUMPLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuadro N.° 1: incompatibilidades por cercanía</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuadro N.° 2: condiciones propias del hogar</t>
   </si>
   <si>
     <t xml:space="preserve">RESULTADO</t>
@@ -368,7 +462,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -383,6 +477,19 @@
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
@@ -417,7 +524,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -451,6 +558,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1326,11 +1437,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1345,46 +1460,190 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="D4" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B5" s="6" t="n">
-        <f aca="false">COUNTA(MATRIZ!B5:B22)</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="E4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF(MATRIZ!H5:H22,"CUMPLE")</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="F4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF(MATRIZ!H5:H22,"NO CUMPLE")</f>
-        <v>0</v>
+      <c r="C5" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F5" s="6" t="str">
+        <f aca="false">IF(D5="SÍ","CUMPLE","NO CUMPLE")</f>
+        <v>CUMPLE</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="6" t="str">
+        <f aca="false">IF(D6="SÍ","CUMPLE","NO CUMPLE")</f>
+        <v>CUMPLE</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" s="6" t="str">
+        <f aca="false">IF(D7="SÍ","CUMPLE","NO CUMPLE")</f>
+        <v>CUMPLE</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="F8" s="6" t="str">
+        <f aca="false">IF(D8="SÍ","CUMPLE","NO CUMPLE")</f>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B9" s="6" t="str">
-        <f aca="false">IF(B7=0,"UBICACIÓN APTA","REVISAR")</f>
-        <v>UBICACIÓN APTA</v>
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" s="6" t="str">
+        <f aca="false">IF(D9="SÍ","CUMPLE","NO CUMPLE")</f>
+        <v>CUMPLE</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F10" s="6" t="str">
+        <f aca="false">IF(D10="SÍ","CUMPLE","NO CUMPLE")</f>
+        <v>CUMPLE</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F11" s="6" t="str">
+        <f aca="false">IF(D11="SÍ","CUMPLE","NO CUMPLE")</f>
+        <v>CUMPLE</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F12" s="6" t="str">
+        <f aca="false">IF(D12="SÍ","CUMPLE","NO CUMPLE")</f>
+        <v>CUMPLE</v>
       </c>
     </row>
   </sheetData>
@@ -1396,4 +1655,99 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <f aca="false">COUNTA(MATRIZ!B5:B22)</f>
+        <v>18</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <f aca="false">COUNTIF(MATRIZ!H5:H22,"CUMPLE")</f>
+        <v>18</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <f aca="false">COUNTIF(MATRIZ!H5:H22,"NO CUMPLE")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <f aca="false">COUNTA('CONDICIONES HOGAR'!B5:B12)</f>
+        <v>8</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <f aca="false">COUNTIF('CONDICIONES HOGAR'!F5:F12,"CUMPLE")</f>
+        <v>8</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <f aca="false">COUNTIF('CONDICIONES HOGAR'!F5:F12,"NO CUMPLE")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" s="9" t="str">
+        <f aca="false">IF(SUM(D5:D6)=0,"TERRENO APTO PARA EL HOGAR DE REFUGIO","REVISAR")</f>
+        <v>TERRENO APTO PARA EL HOGAR DE REFUGIO</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B8:D8"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>